<commit_message>
add native - profiles
</commit_message>
<xml_diff>
--- a/birthday-reader/data/employees.xlsx
+++ b/birthday-reader/data/employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Birthday-Mail\birthday-reader\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C043403D-44F9-457B-B79B-9BD1381A4E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78EEC418-4F73-4FBE-B39E-549317E2C25E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1520" yWindow="1120" windowWidth="15380" windowHeight="8750" xr2:uid="{34D36F85-5268-4715-9CA8-69230E014947}"/>
   </bookViews>
@@ -153,7 +153,7 @@
     <t>13/05/2001</t>
   </si>
   <si>
-    <t>19/05/2000</t>
+    <t>01/06/2000</t>
   </si>
 </sst>
 </file>

</xml_diff>